<commit_message>
Actualizo casos de prueba de solicitud de amistad y gestion de contactos
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas_facebook_lite.xlsx
+++ b/casos_de_prueba/matriz_pruebas_facebook_lite.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4ded0ad4c19a0dfe/Documentos/ProyectoFinal-ToledoMariaEugenia/casos_de_prueba/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C61F0BC8-CEFF-407B-B51E-68E7195793AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{C61F0BC8-CEFF-407B-B51E-68E7195793AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A419965-45A2-4E0B-9AEF-5D96856B3CB4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="278">
   <si>
     <t>Id</t>
   </si>
@@ -514,33 +514,6 @@
     <t>1. Click en 'Agregar amigo'.</t>
   </si>
   <si>
-    <t>1. Ir al perfil. 2. Click en 'Cancelar solicitud'.</t>
-  </si>
-  <si>
-    <t>1. Ir a notificaciones. 2. Click en 'Confirmar'.</t>
-  </si>
-  <si>
-    <t>1. Ir a notificaciones. 2. Click en 'Eliminar'.</t>
-  </si>
-  <si>
-    <t>1. Ir al perfil. 2. Click en 'Amigos'. 3. Elegir 'Eliminar de mis amigos'.</t>
-  </si>
-  <si>
-    <t>1. Ir al perfil propio. 2. Click en 'Ver todos los amigos'.</t>
-  </si>
-  <si>
-    <t>1. Click en menú (...) 2. Elegir 'Bloquear'.</t>
-  </si>
-  <si>
-    <t>1. Ajustes. 2. Bloqueos. 3. Desbloquear.</t>
-  </si>
-  <si>
-    <t>1. Ir a pestaña 'Amigos'. 2. Ver sección 'Sugerencias'.</t>
-  </si>
-  <si>
-    <t>1. Entrar al perfil. 2. Click en 'Seguir'.</t>
-  </si>
-  <si>
     <t>1. Click en Mensaje. 2. Escribir 'Hola'. 3. Enviar.</t>
   </si>
   <si>
@@ -625,19 +598,7 @@
     <t>Ana</t>
   </si>
   <si>
-    <t>Perfil B</t>
-  </si>
-  <si>
     <t>Perfil C</t>
-  </si>
-  <si>
-    <t>Perfil D</t>
-  </si>
-  <si>
-    <t>Amigo E</t>
-  </si>
-  <si>
-    <t>Usuario X</t>
   </si>
   <si>
     <t>Página Pública</t>
@@ -856,6 +817,62 @@
   </si>
   <si>
     <t>No aparece el mensaje de error y la pantalla queda congelada</t>
+  </si>
+  <si>
+    <t>1. Ir al perfil. 
+2. Click en 'Cancelar solicitud'.</t>
+  </si>
+  <si>
+    <t>1. Ir a notificaciones. 
+2. Click en 'Confirmar'.</t>
+  </si>
+  <si>
+    <t>1. Ir a notificaciones. 
+2. Click en 'Eliminar'.</t>
+  </si>
+  <si>
+    <t>1. Ir al perfil. 
+2. Click en 'Amigos'. 
+3. Elegir 'Eliminar de mis amigos'.</t>
+  </si>
+  <si>
+    <t>El botón cambió a 'Cancel request'</t>
+  </si>
+  <si>
+    <t>El botón cambió a 'Friends'</t>
+  </si>
+  <si>
+    <t>No desaparece al instante, hay que refrescar la vista</t>
+  </si>
+  <si>
+    <t>1. Ir al perfil propio. 
+2. Click en 'Ver todos los amigos'.</t>
+  </si>
+  <si>
+    <t>1. Ajustes. 
+2. Bloqueos. 
+3. Desbloquear.</t>
+  </si>
+  <si>
+    <t>1. Ir a pestaña 'Amigos'. 
+2. Ver sección 'Sugerencias'.</t>
+  </si>
+  <si>
+    <t>1. Entrar al perfil. 
+2. Click en 'Seguir'.</t>
+  </si>
+  <si>
+    <t>Mariana Viskup</t>
+  </si>
+  <si>
+    <t>1. Click en los tres puntos (...) 
+2. Elegir 'Bloquear'.</t>
+  </si>
+  <si>
+    <t>Por el momento me figura una sola sugerencia</t>
+  </si>
+  <si>
+    <t>La sugerencia no es pública</t>
   </si>
 </sst>
 </file>
@@ -929,7 +946,24 @@
   <dxfs count="7">
     <dxf>
       <font>
-        <color theme="5"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
       </font>
       <fill>
         <patternFill>
@@ -965,29 +999,12 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
-        <color theme="1"/>
+        <color theme="5"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="6" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.59996337778862885"/>
+          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1333,7 +1350,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>272</v>
+        <v>259</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -1359,28 +1376,28 @@
         <v>131</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="F2" t="s">
-        <v>265</v>
+        <v>252</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>273</v>
+        <v>260</v>
       </c>
       <c r="J2" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K2" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="L2" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1397,26 +1414,26 @@
         <v>132</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="F3" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>217</v>
+        <v>204</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K3" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L3" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -1433,28 +1450,28 @@
         <v>132</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="F4" t="s">
+        <v>185</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F4" t="s">
-        <v>194</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>274</v>
-      </c>
       <c r="J4" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K4" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L4" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1471,26 +1488,26 @@
         <v>133</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="F5" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K5" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L5" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1507,26 +1524,26 @@
         <v>133</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>263</v>
+        <v>250</v>
       </c>
       <c r="F6" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K6" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L6" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.3">
@@ -1546,23 +1563,23 @@
         <v>160</v>
       </c>
       <c r="F7" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>221</v>
+        <v>208</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K7" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L7" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1579,23 +1596,23 @@
         <v>132</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>269</v>
+        <v>256</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>222</v>
+        <v>209</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K8" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L8" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -1612,26 +1629,26 @@
         <v>134</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>270</v>
+        <v>257</v>
       </c>
       <c r="F9" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>223</v>
+        <v>210</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K9" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L9" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1651,23 +1668,23 @@
         <v>161</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>224</v>
+        <v>211</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K10" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L10" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -1687,28 +1704,28 @@
         <v>162</v>
       </c>
       <c r="F11" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>271</v>
+        <v>258</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>275</v>
+        <v>262</v>
       </c>
       <c r="J11" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K11" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L11" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1725,19 +1742,25 @@
         <v>163</v>
       </c>
       <c r="F12" t="s">
-        <v>201</v>
+        <v>274</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>225</v>
+        <v>212</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>267</v>
       </c>
       <c r="J12" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K12" t="s">
-        <v>258</v>
+        <v>245</v>
       </c>
       <c r="L12" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1754,22 +1777,28 @@
         <v>137</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>164</v>
+        <v>263</v>
       </c>
       <c r="F13" t="s">
-        <v>201</v>
+        <v>274</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>226</v>
+        <v>213</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>268</v>
       </c>
       <c r="J13" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K13" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L13" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1786,25 +1815,28 @@
         <v>138</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>165</v>
+        <v>264</v>
       </c>
       <c r="F14" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>227</v>
+        <v>214</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>255</v>
       </c>
       <c r="J14" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K14" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="L14" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1818,25 +1850,31 @@
         <v>138</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>166</v>
+        <v>265</v>
       </c>
       <c r="F15" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>228</v>
+        <v>215</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>269</v>
       </c>
       <c r="J15" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K15" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L15" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1850,22 +1888,22 @@
         <v>139</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>167</v>
+        <v>266</v>
       </c>
       <c r="F16" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>229</v>
+        <v>216</v>
       </c>
       <c r="J16" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K16" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L16" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1882,25 +1920,28 @@
         <v>140</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>168</v>
+        <v>270</v>
       </c>
       <c r="F17" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>230</v>
+        <v>217</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>255</v>
       </c>
       <c r="J17" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K17" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L17" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -1914,25 +1955,28 @@
         <v>136</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>169</v>
+        <v>275</v>
       </c>
       <c r="F18" t="s">
-        <v>205</v>
+        <v>274</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>231</v>
+        <v>218</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>255</v>
       </c>
       <c r="J18" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K18" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="L18" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1946,25 +1990,28 @@
         <v>141</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>170</v>
+        <v>271</v>
       </c>
       <c r="F19" t="s">
-        <v>205</v>
+        <v>274</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>232</v>
+        <v>219</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>255</v>
       </c>
       <c r="J19" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K19" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L19" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -1978,25 +2025,31 @@
         <v>142</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>171</v>
+        <v>272</v>
       </c>
       <c r="F20" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>233</v>
+        <v>220</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>276</v>
       </c>
       <c r="J20" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K20" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L20" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -2010,22 +2063,28 @@
         <v>143</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>172</v>
+        <v>273</v>
       </c>
       <c r="F21" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>234</v>
+        <v>221</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>277</v>
       </c>
       <c r="J21" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K21" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L21" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2042,22 +2101,22 @@
         <v>144</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="F22" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>235</v>
+        <v>222</v>
       </c>
       <c r="J22" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K22" t="s">
-        <v>258</v>
+        <v>245</v>
       </c>
       <c r="L22" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2074,22 +2133,22 @@
         <v>132</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="F23" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>236</v>
+        <v>223</v>
       </c>
       <c r="J23" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K23" t="s">
-        <v>258</v>
+        <v>245</v>
       </c>
       <c r="L23" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
@@ -2106,22 +2165,22 @@
         <v>145</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="F24" t="s">
-        <v>208</v>
+        <v>195</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>237</v>
+        <v>224</v>
       </c>
       <c r="J24" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K24" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L24" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2138,22 +2197,22 @@
         <v>146</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="F25" t="s">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>238</v>
+        <v>225</v>
       </c>
       <c r="J25" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K25" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="L25" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
@@ -2170,22 +2229,22 @@
         <v>147</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="F26" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>239</v>
+        <v>226</v>
       </c>
       <c r="J26" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K26" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L26" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2202,22 +2261,22 @@
         <v>148</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="F27" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>240</v>
+        <v>227</v>
       </c>
       <c r="J27" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K27" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L27" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2234,22 +2293,22 @@
         <v>149</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="F28" t="s">
-        <v>210</v>
+        <v>197</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>241</v>
+        <v>228</v>
       </c>
       <c r="J28" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K28" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="L28" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2266,22 +2325,22 @@
         <v>150</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="F29" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>242</v>
+        <v>229</v>
       </c>
       <c r="J29" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K29" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L29" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2298,22 +2357,22 @@
         <v>151</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="F30" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>243</v>
+        <v>230</v>
       </c>
       <c r="J30" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K30" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L30" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
@@ -2330,22 +2389,22 @@
         <v>152</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="F31" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>244</v>
+        <v>231</v>
       </c>
       <c r="J31" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K31" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="L31" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
@@ -2362,22 +2421,22 @@
         <v>153</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="F32" t="s">
-        <v>213</v>
+        <v>200</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>245</v>
+        <v>232</v>
       </c>
       <c r="J32" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K32" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="L32" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2394,22 +2453,22 @@
         <v>154</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="F33" t="s">
-        <v>214</v>
+        <v>201</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>246</v>
+        <v>233</v>
       </c>
       <c r="J33" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K33" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L33" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
@@ -2426,22 +2485,22 @@
         <v>155</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="F34" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="J34" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K34" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="L34" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2458,22 +2517,22 @@
         <v>156</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="F35" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>248</v>
+        <v>235</v>
       </c>
       <c r="J35" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K35" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L35" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2490,22 +2549,22 @@
         <v>157</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="F36" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>249</v>
+        <v>236</v>
       </c>
       <c r="J36" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="K36" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L36" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
@@ -2522,22 +2581,22 @@
         <v>155</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="F37" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>250</v>
+        <v>237</v>
       </c>
       <c r="J37" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K37" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L37" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
@@ -2554,22 +2613,22 @@
         <v>155</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="F38" t="s">
-        <v>216</v>
+        <v>203</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>251</v>
+        <v>238</v>
       </c>
       <c r="J38" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K38" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L38" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
@@ -2586,22 +2645,22 @@
         <v>158</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="F39" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>252</v>
+        <v>239</v>
       </c>
       <c r="J39" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K39" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="L39" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="40" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2618,22 +2677,22 @@
         <v>158</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="F40" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>253</v>
+        <v>240</v>
       </c>
       <c r="J40" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K40" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L40" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2650,33 +2709,38 @@
         <v>159</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="F41" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="J41" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="K41" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="L41" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:I41">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="FAIL">
+  <conditionalFormatting sqref="H2:I2">
+    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="FAIL">
       <formula>NOT(ISERROR(SEARCH("FAIL",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="OK">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:I41">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="FAIL">
+      <formula>NOT(ISERROR(SEARCH("FAIL",H2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="OK">
+    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",H2)))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="5">
@@ -2688,11 +2752,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:I2">
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="FAIL">
-      <formula>NOT(ISERROR(SEARCH("FAIL",H2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sumo nuevas capturas como evidencia de las pruebas funcionales
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas_facebook_lite.xlsx
+++ b/casos_de_prueba/matriz_pruebas_facebook_lite.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="36" documentId="8_{C61F0BC8-CEFF-407B-B51E-68E7195793AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A419965-45A2-4E0B-9AEF-5D96856B3CB4}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -943,34 +943,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <font>
         <color theme="1"/>
@@ -2729,18 +2702,18 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H2:I2">
-    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="FAIL">
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="FAIL">
       <formula>NOT(ISERROR(SEARCH("FAIL",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:I41">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="FAIL">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="FAIL">
       <formula>NOT(ISERROR(SEARCH("FAIL",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="OK">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="OK">
+    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",H2)))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="5">

</xml_diff>

<commit_message>
Agrego nuevos casos ejecutados con sus respectivas evidencias. Inicio de conversaciones y gestión de contactos
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas_facebook_lite.xlsx
+++ b/casos_de_prueba/matriz_pruebas_facebook_lite.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4ded0ad4c19a0dfe/Documentos/ProyectoFinal-ToledoMariaEugenia/casos_de_prueba/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{C61F0BC8-CEFF-407B-B51E-68E7195793AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A419965-45A2-4E0B-9AEF-5D96856B3CB4}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="8_{C61F0BC8-CEFF-407B-B51E-68E7195793AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC780216-FA74-4380-A004-923048C05572}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="281">
   <si>
     <t>Id</t>
   </si>
@@ -514,33 +514,9 @@
     <t>1. Click en 'Agregar amigo'.</t>
   </si>
   <si>
-    <t>1. Click en Mensaje. 2. Escribir 'Hola'. 3. Enviar.</t>
-  </si>
-  <si>
-    <t>1. Recibir mensaje de un tercero. 2. Abrir notificación.</t>
-  </si>
-  <si>
-    <t>1. Seleccionar emoji. 2. Enviar.</t>
-  </si>
-  <si>
-    <t>1. Click en ícono cámara/galería. 2. Elegir foto. 3. Enviar.</t>
-  </si>
-  <si>
     <t>1. Esperar a que el otro usuario lea.</t>
   </si>
   <si>
-    <t>1. Mantener presionado mensaje. 2. Click 'Eliminar para todos'.</t>
-  </si>
-  <si>
-    <t>1. Nuevo mensaje. 2. Seleccionar 2 amigos. 3. Enviar mensaje inicial.</t>
-  </si>
-  <si>
-    <t>1. Abrir chat. 2. Configuración. 3. Silenciar.</t>
-  </si>
-  <si>
-    <t>1. Opciones de chat. 2. Buscar. 3. Escribir palabra.</t>
-  </si>
-  <si>
     <t>1. Enviar mensaje corto.</t>
   </si>
   <si>
@@ -598,9 +574,6 @@
     <t>Ana</t>
   </si>
   <si>
-    <t>Perfil C</t>
-  </si>
-  <si>
     <t>Página Pública</t>
   </si>
   <si>
@@ -611,9 +584,6 @@
   </si>
   <si>
     <t>Imagen .jpg</t>
-  </si>
-  <si>
-    <t>Amigo A + B</t>
   </si>
   <si>
     <t>'Reunión'</t>
@@ -873,6 +843,59 @@
   </si>
   <si>
     <t>La sugerencia no es pública</t>
+  </si>
+  <si>
+    <t>1. Click en Mensaje. 
+2. Escribir 'Hola'. 
+3. Enviar.</t>
+  </si>
+  <si>
+    <t>1. Recibir mensaje de un tercero. 
+2. Abrir notificación.</t>
+  </si>
+  <si>
+    <t>1. Seleccionar emoji. 
+2. Enviar.</t>
+  </si>
+  <si>
+    <t>1. Click en ícono cámara/galería. 
+2. Elegir foto. 
+3. Enviar.</t>
+  </si>
+  <si>
+    <t>1. Mantener presionado mensaje. 
+2. Click 'Eliminar para todos'.</t>
+  </si>
+  <si>
+    <t>No aparece el mensaje o el tag de 'Leido', figura la foto del usuario al lado del mensaje como leído</t>
+  </si>
+  <si>
+    <t>Eugenia Toledo + Cecilia Toledo</t>
+  </si>
+  <si>
+    <t>Eugenia Toledo</t>
+  </si>
+  <si>
+    <t>1. Opciones de chat. 
+2. Buscar. 
+3. Escribir palabra.</t>
+  </si>
+  <si>
+    <t>1. Nuevo mensaje. 
+2. Seleccionar 2 amigos. 
+3. Enviar mensaje inicial 'Hola'.</t>
+  </si>
+  <si>
+    <t>1. Abrir chat. 
+2. Configuración. 
+3. Silenciar.
+4. Silenciar por 15 minutos.</t>
+  </si>
+  <si>
+    <t>BLOQUEADO</t>
+  </si>
+  <si>
+    <t>La ejecución de estas pruebas se realizó en una tablet de android ya que no cuento con dispositivo movil con dicho SO</t>
   </si>
 </sst>
 </file>
@@ -943,7 +966,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="1"/>
@@ -1323,7 +1356,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -1349,28 +1382,28 @@
         <v>131</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="F2" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="J2" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K2" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="L2" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1387,26 +1420,26 @@
         <v>132</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="F3" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K3" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L3" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -1423,28 +1456,28 @@
         <v>132</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="F4" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="J4" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K4" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L4" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1461,26 +1494,26 @@
         <v>133</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="F5" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K5" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L5" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1497,26 +1530,26 @@
         <v>133</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="F6" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K6" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L6" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.3">
@@ -1536,23 +1569,23 @@
         <v>160</v>
       </c>
       <c r="F7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K7" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L7" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1569,23 +1602,23 @@
         <v>132</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K8" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L8" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -1602,26 +1635,26 @@
         <v>134</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="F9" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K9" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L9" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1641,23 +1674,23 @@
         <v>161</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K10" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L10" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -1677,25 +1710,25 @@
         <v>162</v>
       </c>
       <c r="F11" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="J11" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K11" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L11" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1715,25 +1748,25 @@
         <v>163</v>
       </c>
       <c r="F12" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="J12" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K12" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="L12" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1750,28 +1783,28 @@
         <v>137</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="F13" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="J13" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K13" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L13" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1788,25 +1821,25 @@
         <v>138</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="F14" t="s">
-        <v>192</v>
+        <v>275</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="J14" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K14" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="L14" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -1823,28 +1856,28 @@
         <v>138</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="F15" t="s">
-        <v>192</v>
+        <v>275</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="J15" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K15" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L15" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -1861,22 +1894,25 @@
         <v>139</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="F16" t="s">
-        <v>192</v>
+        <v>275</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>216</v>
+        <v>206</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="J16" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K16" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L16" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1893,25 +1929,25 @@
         <v>140</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="F17" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="J17" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K17" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L17" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1928,25 +1964,25 @@
         <v>136</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="F18" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="J18" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K18" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="L18" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -1963,25 +1999,25 @@
         <v>141</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="F19" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="J19" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K19" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L19" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -1998,28 +2034,28 @@
         <v>142</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="F20" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="J20" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K20" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L20" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2036,31 +2072,31 @@
         <v>143</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="F21" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="J21" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K21" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L21" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -2074,22 +2110,25 @@
         <v>144</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>164</v>
+        <v>268</v>
       </c>
       <c r="F22" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>222</v>
+        <v>212</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="J22" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K22" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="L22" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2106,25 +2145,28 @@
         <v>132</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>165</v>
+        <v>269</v>
       </c>
       <c r="F23" t="s">
-        <v>189</v>
+        <v>275</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>223</v>
+        <v>213</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="J23" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K23" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="L23" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>33</v>
       </c>
@@ -2138,25 +2180,28 @@
         <v>145</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>166</v>
+        <v>270</v>
       </c>
       <c r="F24" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>224</v>
+        <v>214</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="J24" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K24" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L24" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -2170,25 +2215,28 @@
         <v>146</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>167</v>
+        <v>271</v>
       </c>
       <c r="F25" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>225</v>
+        <v>215</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="J25" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K25" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="L25" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -2202,22 +2250,28 @@
         <v>147</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="F26" t="s">
-        <v>189</v>
+        <v>275</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>226</v>
+        <v>216</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>273</v>
       </c>
       <c r="J26" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K26" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L26" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2234,25 +2288,28 @@
         <v>148</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>169</v>
+        <v>272</v>
       </c>
       <c r="F27" t="s">
-        <v>189</v>
+        <v>275</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>227</v>
+        <v>217</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="J27" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K27" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L27" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -2266,25 +2323,28 @@
         <v>149</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="F28" t="s">
-        <v>197</v>
+        <v>277</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>274</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>228</v>
+        <v>218</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="J28" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K28" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="L28" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -2298,25 +2358,28 @@
         <v>150</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>171</v>
+        <v>278</v>
       </c>
       <c r="F29" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>229</v>
+        <v>219</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="J29" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K29" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L29" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>39</v>
       </c>
@@ -2330,25 +2393,31 @@
         <v>151</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>172</v>
+        <v>276</v>
       </c>
       <c r="F30" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>230</v>
+        <v>220</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>280</v>
       </c>
       <c r="J30" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K30" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L30" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>40</v>
       </c>
@@ -2362,22 +2431,28 @@
         <v>152</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="F31" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>231</v>
+        <v>221</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>280</v>
       </c>
       <c r="J31" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K31" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="L31" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
@@ -2394,22 +2469,22 @@
         <v>153</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="F32" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="G32" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="J32" t="s">
         <v>232</v>
       </c>
-      <c r="J32" t="s">
-        <v>242</v>
-      </c>
       <c r="K32" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="L32" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2426,22 +2501,22 @@
         <v>154</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="F33" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="J33" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K33" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L33" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
@@ -2458,22 +2533,22 @@
         <v>155</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="F34" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="J34" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K34" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="L34" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2490,22 +2565,22 @@
         <v>156</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="F35" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="J35" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K35" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L35" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2522,22 +2597,22 @@
         <v>157</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="F36" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="J36" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="K36" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L36" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
@@ -2554,22 +2629,22 @@
         <v>155</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="F37" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="J37" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K37" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L37" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
@@ -2586,22 +2661,22 @@
         <v>155</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="F38" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="J38" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K38" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L38" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
@@ -2618,22 +2693,22 @@
         <v>158</v>
       </c>
       <c r="E39" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F39" t="s">
         <v>181</v>
       </c>
-      <c r="F39" t="s">
-        <v>189</v>
-      </c>
       <c r="G39" s="2" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="J39" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K39" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="L39" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="40" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2650,22 +2725,22 @@
         <v>158</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="F40" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="J40" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="K40" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L40" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -2682,41 +2757,41 @@
         <v>159</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="F41" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="J41" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K41" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="L41" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H2:I2">
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="FAIL">
+    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="FAIL">
       <formula>NOT(ISERROR(SEARCH("FAIL",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:I41">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="FAIL">
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="FAIL">
       <formula>NOT(ISERROR(SEARCH("FAIL",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="OK">
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="OK">
+    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",H2)))</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2725,6 +2800,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H41">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="BLOQUEADO">
+      <formula>NOT(ISERROR(SEARCH("BLOQUEADO",H2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sumo word del informe final
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas_facebook_lite.xlsx
+++ b/casos_de_prueba/matriz_pruebas_facebook_lite.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4ded0ad4c19a0dfe/Documentos/ProyectoFinal-ToledoMariaEugenia/casos_de_prueba/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="108" documentId="8_{C61F0BC8-CEFF-407B-B51E-68E7195793AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9086786B-2384-44D2-B8DC-1E094D642EF4}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="8_{C61F0BC8-CEFF-407B-B51E-68E7195793AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E607A34D-7909-4200-BBE4-30B9E7E207A3}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="31425" yWindow="3075" windowWidth="21345" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1074,10 +1074,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2446,7 +2442,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>39</v>
       </c>
@@ -2484,7 +2480,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>40</v>
       </c>
@@ -2888,6 +2884,7 @@
   <autoFilter ref="A1:L41" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="7">
       <filters>
+        <filter val="BLOQUEADO"/>
         <filter val="FAIL"/>
       </filters>
     </filterColumn>

</xml_diff>